<commit_message>
modificato report-checklist.xlsx come richiesto
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111CIDITECHSRLXX/Ciditech/Point/9.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111CIDITECHSRLXX/Ciditech/Point/9.0/report-checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antonio\Documents\FSE Lombardia\it-fse-accreditamento\GATEWAY\A1#111CIDITECHSRLXX\Ciditech\Point\9.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7367783-6B51-4A71-A395-D0CB750BB390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4277650F-E7D0-4512-B911-CFFD1FFF15B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="241">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -1000,7 +1000,7 @@
     <numFmt numFmtId="165" formatCode="d/m/yyyy\ hh:mm:ss"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1128,6 +1128,28 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1467,7 +1489,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1624,6 +1646,11 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal 2" xfId="1" xr:uid="{565105C8-FFD6-432C-8B2E-BD1D172FCD26}"/>
@@ -3062,7 +3089,6 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:W605"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3188,10 +3214,10 @@
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="59"/>
       <c r="B5" s="60"/>
-      <c r="C5" s="61" t="s">
+      <c r="C5" s="63" t="s">
         <v>171</v>
       </c>
-      <c r="D5" s="53"/>
+      <c r="D5" s="64"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -3215,6 +3241,7 @@
       <c r="A6" s="50"/>
       <c r="B6" s="51"/>
       <c r="C6" s="10"/>
+      <c r="E6" s="62"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -3348,7 +3375,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="33">
         <v>29</v>
       </c>
@@ -3409,7 +3436,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="33">
         <v>32</v>
       </c>
@@ -3470,7 +3497,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="33">
         <v>37</v>
       </c>
@@ -3531,7 +3558,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="33">
         <v>40</v>
       </c>
@@ -3592,7 +3619,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="33">
         <v>45</v>
       </c>
@@ -3651,7 +3678,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="33">
         <v>48</v>
       </c>
@@ -3710,7 +3737,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="33">
         <v>64</v>
       </c>
@@ -3771,7 +3798,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33">
         <v>66</v>
       </c>
@@ -3808,7 +3835,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="33">
         <v>67</v>
       </c>
@@ -3869,7 +3896,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="33">
         <v>68</v>
       </c>
@@ -3930,7 +3957,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="33">
         <v>69</v>
       </c>
@@ -3991,7 +4018,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="33">
         <v>70</v>
       </c>
@@ -4051,7 +4078,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="33">
         <v>71</v>
       </c>
@@ -4092,7 +4119,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="33">
         <v>72</v>
       </c>
@@ -4133,7 +4160,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="33">
         <v>73</v>
       </c>
@@ -4194,7 +4221,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="33">
         <v>74</v>
       </c>
@@ -4235,7 +4262,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="26" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="33">
         <v>152</v>
       </c>
@@ -4296,7 +4323,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="27" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="33">
         <v>154</v>
       </c>
@@ -4337,7 +4364,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="28" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="33">
         <v>155</v>
       </c>
@@ -4398,7 +4425,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="33">
         <v>156</v>
       </c>
@@ -4459,7 +4486,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="30" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="33">
         <v>159</v>
       </c>
@@ -4500,7 +4527,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="31" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="33">
         <v>160</v>
       </c>
@@ -4561,7 +4588,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="32" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="33">
         <v>161</v>
       </c>
@@ -4622,7 +4649,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="33" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="33">
         <v>162</v>
       </c>
@@ -4683,7 +4710,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="34" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="33">
         <v>163</v>
       </c>
@@ -4744,7 +4771,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="33">
         <v>164</v>
       </c>
@@ -4785,7 +4812,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="33">
         <v>165</v>
       </c>
@@ -4826,7 +4853,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="33">
         <v>166</v>
       </c>
@@ -4867,7 +4894,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="33">
         <v>167</v>
       </c>
@@ -4908,7 +4935,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="33">
         <v>168</v>
       </c>
@@ -4949,7 +4976,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="33">
         <v>169</v>
       </c>
@@ -5026,16 +5053,22 @@
       <c r="E41" s="40" t="s">
         <v>140</v>
       </c>
-      <c r="F41" s="34"/>
-      <c r="G41" s="44"/>
-      <c r="H41" s="34"/>
-      <c r="I41" s="39"/>
+      <c r="F41" s="34">
+        <v>46090</v>
+      </c>
+      <c r="G41" s="44">
+        <v>46090.459652777776</v>
+      </c>
+      <c r="H41" s="34" t="s">
+        <v>239</v>
+      </c>
+      <c r="I41" s="39" t="s">
+        <v>240</v>
+      </c>
       <c r="J41" s="35" t="s">
-        <v>89</v>
-      </c>
-      <c r="K41" s="35" t="s">
-        <v>92</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="K41" s="35"/>
       <c r="L41" s="35"/>
       <c r="M41" s="35"/>
       <c r="N41" s="35"/>
@@ -5044,7 +5077,9 @@
       <c r="Q41" s="35"/>
       <c r="R41" s="35"/>
       <c r="S41" s="35"/>
-      <c r="T41" s="35"/>
+      <c r="T41" s="35" t="s">
+        <v>87</v>
+      </c>
       <c r="U41" s="36"/>
       <c r="V41" s="37"/>
       <c r="W41" s="35" t="s">
@@ -5067,22 +5102,12 @@
       <c r="E42" s="40" t="s">
         <v>141</v>
       </c>
-      <c r="F42" s="34">
-        <v>46090</v>
-      </c>
-      <c r="G42" s="44">
-        <v>46090.459652777776</v>
-      </c>
-      <c r="H42" s="34" t="s">
-        <v>239</v>
-      </c>
-      <c r="I42" s="39" t="s">
-        <v>240</v>
-      </c>
       <c r="J42" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="K42" s="35"/>
+        <v>89</v>
+      </c>
+      <c r="K42" s="35" t="s">
+        <v>92</v>
+      </c>
       <c r="L42" s="35"/>
       <c r="M42" s="35"/>
       <c r="N42" s="35"/>
@@ -5091,9 +5116,6 @@
       <c r="Q42" s="35"/>
       <c r="R42" s="35"/>
       <c r="S42" s="35"/>
-      <c r="T42" s="35" t="s">
-        <v>87</v>
-      </c>
       <c r="U42" s="36"/>
       <c r="V42" s="37"/>
       <c r="W42" s="35" t="s">
@@ -5210,7 +5232,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="45" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="33">
         <v>461</v>
       </c>
@@ -5251,7 +5273,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="33">
         <v>467</v>
       </c>
@@ -5300,7 +5322,9 @@
         <v>89</v>
       </c>
       <c r="R46" s="35"/>
-      <c r="S46" s="33"/>
+      <c r="S46" s="35" t="s">
+        <v>198</v>
+      </c>
       <c r="T46" s="35" t="s">
         <v>87</v>
       </c>
@@ -5310,7 +5334,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="33">
         <v>468</v>
       </c>
@@ -5351,7 +5375,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="92.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:23" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="33">
         <v>475</v>
       </c>
@@ -9357,13 +9381,7 @@
     <row r="604" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="605" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A9:W48" xr:uid="{00000000-0001-0000-0200-000000000000}">
-    <filterColumn colId="22">
-      <filters>
-        <filter val="OK"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A9:W48" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <mergeCells count="7">
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A2:B2"/>
@@ -9386,17 +9404,17 @@
           </x14:formula1>
           <xm:sqref>M10:N48 P10:R48 J10:J48</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{70793024-27E9-4E6A-BACD-083AB683BC38}">
-          <x14:formula1>
-            <xm:f>Sheet1!$A$2:$A$3</xm:f>
-          </x14:formula1>
-          <xm:sqref>T10:T48</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3DE61C5E-9DA3-4CE3-A1FF-8FBE651EA6B5}">
           <x14:formula1>
             <xm:f>'LISTA VALORI'!$A$2:$A$8</xm:f>
           </x14:formula1>
           <xm:sqref>K10:K20 K22:K48</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{70793024-27E9-4E6A-BACD-083AB683BC38}">
+          <x14:formula1>
+            <xm:f>Sheet1!$A$2:$A$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>T43:T48 T10:T41</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -11633,6 +11651,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BE9A258ADBC3EC4CBEB1E2AB9909207A" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0284f501378927579289f00316ec8a74">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="295b7897-c886-40bf-9750-5782b814c3e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b47213d65be806e283915cff374a7eef" ns2:_="">
     <xsd:import namespace="295b7897-c886-40bf-9750-5782b814c3e4"/>
@@ -11776,22 +11809,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7568E770-0BC4-46AF-B6C6-958AE21C8F7F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11809,31 +11852,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{e0793d39-0939-496d-b129-198edd916feb}" enabled="0" method="" siteId="{e0793d39-0939-496d-b129-198edd916feb}" removed="1"/>

</xml_diff>

<commit_message>
inserito test 451 mancante
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111CIDITECHSRLXX/Ciditech/Point/9.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111CIDITECHSRLXX/Ciditech/Point/9.0/report-checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antonio\Documents\FSE Lombardia\it-fse-accreditamento\GATEWAY\A1#111CIDITECHSRLXX\Ciditech\Point\9.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B48783C-62A7-4DBF-B9D7-4D46AB3B2AB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D025619-DDAB-43D6-A6DD-8D14FBE76C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2805" yWindow="1500" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="239">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -958,9 +958,6 @@
     <t>Errore semantico: [ERRORE-30| L'elemento ClinicalDocument/legalAuthenticator/signatureCode deve essere valorizzato con il codice \"S\" ]</t>
   </si>
   <si>
-    <t>Errore semantico: [ERRORE-b1| Sezione Prestazioni: la sezione DEVE essere presente]</t>
-  </si>
-  <si>
     <t>87c75abe38f5b97f376e66846b259932</t>
   </si>
   <si>
@@ -980,6 +977,12 @@
   </si>
   <si>
     <t>2.16.840.1.113883.2.9.2.10.639.4.4.b738acf04f7eccafb1ae9e8a092932b0f8ff927c9d67b93a2aabe9396ed57c0e.bd85fd14ea^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>a50838f6cae803858d9804c56d305b9f</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.d2b1aca57ee481f1a79c7646e943a39ff77240b1dadc0a0c463b0b0739f35e1f.93d8e44eab^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -5091,10 +5094,10 @@
         <v>46090.459652777776</v>
       </c>
       <c r="H41" s="34" t="s">
+        <v>235</v>
+      </c>
+      <c r="I41" s="39" t="s">
         <v>236</v>
-      </c>
-      <c r="I41" s="39" t="s">
-        <v>237</v>
       </c>
       <c r="J41" s="35" t="s">
         <v>51</v>
@@ -5170,43 +5173,29 @@
         <v>136</v>
       </c>
       <c r="F43" s="34">
-        <v>46085</v>
+        <v>46098</v>
       </c>
       <c r="G43" s="44">
-        <v>46085.494710648149</v>
+        <v>46098.422615740739</v>
       </c>
       <c r="H43" s="34" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="I43" s="39" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="J43" s="35" t="s">
         <v>51</v>
       </c>
       <c r="K43" s="35"/>
       <c r="L43" s="35"/>
-      <c r="M43" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="N43" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="O43" s="35" t="s">
-        <v>230</v>
-      </c>
-      <c r="P43" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q43" s="35" t="s">
-        <v>89</v>
-      </c>
-      <c r="R43" s="35" t="s">
-        <v>89</v>
-      </c>
-      <c r="S43" s="35" t="s">
-        <v>198</v>
-      </c>
+      <c r="M43" s="35"/>
+      <c r="N43" s="35"/>
+      <c r="O43" s="35"/>
+      <c r="P43" s="35"/>
+      <c r="Q43" s="35"/>
+      <c r="R43" s="35"/>
+      <c r="S43" s="35"/>
       <c r="T43" s="35" t="s">
         <v>87</v>
       </c>
@@ -5239,10 +5228,10 @@
         <v>46085.56591435185</v>
       </c>
       <c r="H44" s="34" t="s">
+        <v>230</v>
+      </c>
+      <c r="I44" s="39" t="s">
         <v>231</v>
-      </c>
-      <c r="I44" s="39" t="s">
-        <v>232</v>
       </c>
       <c r="J44" s="35" t="s">
         <v>51</v>
@@ -5329,10 +5318,10 @@
         <v>46085.563715277778</v>
       </c>
       <c r="H46" s="35" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="I46" s="35" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J46" s="35" t="s">
         <v>51</v>
@@ -5346,7 +5335,7 @@
         <v>51</v>
       </c>
       <c r="O46" s="35" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="P46" s="35" t="s">
         <v>51</v>
@@ -11678,6 +11667,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BE9A258ADBC3EC4CBEB1E2AB9909207A" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0284f501378927579289f00316ec8a74">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="295b7897-c886-40bf-9750-5782b814c3e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b47213d65be806e283915cff374a7eef" ns2:_="">
     <xsd:import namespace="295b7897-c886-40bf-9750-5782b814c3e4"/>
@@ -11821,22 +11825,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7568E770-0BC4-46AF-B6C6-958AE21C8F7F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11854,31 +11868,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{e0793d39-0939-496d-b129-198edd916feb}" enabled="0" method="" siteId="{e0793d39-0939-496d-b129-198edd916feb}" removed="1"/>

</xml_diff>

<commit_message>
fix test 451 e id nel json
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111CIDITECHSRLXX/Ciditech/Point/9.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111CIDITECHSRLXX/Ciditech/Point/9.0/report-checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antonio\Documents\FSE Lombardia\it-fse-accreditamento\GATEWAY\A1#111CIDITECHSRLXX\Ciditech\Point\9.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D025619-DDAB-43D6-A6DD-8D14FBE76C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87DEE500-CC80-4662-836A-EA6ACECAB374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2805" yWindow="1500" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3840" yWindow="2535" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="240">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -958,12 +958,6 @@
     <t>Errore semantico: [ERRORE-30| L'elemento ClinicalDocument/legalAuthenticator/signatureCode deve essere valorizzato con il codice \"S\" ]</t>
   </si>
   <si>
-    <t>87c75abe38f5b97f376e66846b259932</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.a55f567080dde90eb939ce3a18a0a952f87b2f35411df25e15aa44509bf3b1ec.ccc6b5d3a7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>5f826dbfc669c773409b317611f1c7f3</t>
   </si>
   <si>
@@ -983,6 +977,15 @@
   </si>
   <si>
     <t>2.16.840.1.113883.2.9.2.10.639.4.4.d2b1aca57ee481f1a79c7646e943a39ff77240b1dadc0a0c463b0b0739f35e1f.93d8e44eab^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>18/03/2026 110327</t>
+  </si>
+  <si>
+    <t>0c7ef65713fd9e5516762ca869f246da</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.a55f567080dde90eb939ce3a18a0a952f87b2f35411df25e15aa44509bf3b1ec.1a1b850998^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -5094,10 +5097,10 @@
         <v>46090.459652777776</v>
       </c>
       <c r="H41" s="34" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="I41" s="39" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="J41" s="35" t="s">
         <v>51</v>
@@ -5179,10 +5182,10 @@
         <v>46098.422615740739</v>
       </c>
       <c r="H43" s="34" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="I43" s="39" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="J43" s="35" t="s">
         <v>51</v>
@@ -5222,16 +5225,16 @@
         <v>137</v>
       </c>
       <c r="F44" s="34">
-        <v>46085</v>
-      </c>
-      <c r="G44" s="44">
-        <v>46085.56591435185</v>
+        <v>46099</v>
+      </c>
+      <c r="G44" s="44" t="s">
+        <v>237</v>
       </c>
       <c r="H44" s="34" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="I44" s="39" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="J44" s="35" t="s">
         <v>51</v>
@@ -5318,10 +5321,10 @@
         <v>46085.563715277778</v>
       </c>
       <c r="H46" s="35" t="s">
+        <v>230</v>
+      </c>
+      <c r="I46" s="35" t="s">
         <v>232</v>
-      </c>
-      <c r="I46" s="35" t="s">
-        <v>234</v>
       </c>
       <c r="J46" s="35" t="s">
         <v>51</v>
@@ -5335,7 +5338,7 @@
         <v>51</v>
       </c>
       <c r="O46" s="35" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="P46" s="35" t="s">
         <v>51</v>
@@ -11673,15 +11676,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BE9A258ADBC3EC4CBEB1E2AB9909207A" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0284f501378927579289f00316ec8a74">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="295b7897-c886-40bf-9750-5782b814c3e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b47213d65be806e283915cff374a7eef" ns2:_="">
     <xsd:import namespace="295b7897-c886-40bf-9750-5782b814c3e4"/>
@@ -11825,6 +11819,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
   <ds:schemaRefs>
@@ -11843,14 +11846,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7568E770-0BC4-46AF-B6C6-958AE21C8F7F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11868,6 +11863,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{e0793d39-0939-496d-b129-198edd916feb}" enabled="0" method="" siteId="{e0793d39-0939-496d-b129-198edd916feb}" removed="1"/>

</xml_diff>

<commit_message>
rifatti tutti i test per i dati mancanti
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111CIDITECHSRLXX/Ciditech/Point/9.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111CIDITECHSRLXX/Ciditech/Point/9.0/report-checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antonio\Documents\FSE Lombardia\it-fse-accreditamento\GATEWAY\A1#111CIDITECHSRLXX\Ciditech\Point\9.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87DEE500-CC80-4662-836A-EA6ACECAB374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26789A86-9D78-4D4E-8004-6F31180D0C42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3840" yWindow="2535" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="239">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -787,9 +787,6 @@
     <t>subject_application_id: Point</t>
   </si>
   <si>
-    <t>1068c57d9715eee3b25876cf5c4e0353</t>
-  </si>
-  <si>
     <t>UNKNOWN_WORKFLOW_ID</t>
   </si>
   <si>
@@ -799,45 +796,24 @@
     <t>Campo token JWT non valido: Il campo action_id non è corretto</t>
   </si>
   <si>
-    <t>2f9d7a42920e2d6e5c5cf1a91c56e0ba</t>
-  </si>
-  <si>
     <t>Campo token JWT non valido.: Il campo action_id non è corretto</t>
   </si>
   <si>
-    <t>75452e5238d7a55beff8cb3434d05fd4</t>
-  </si>
-  <si>
     <t>Campo token JWT non valido: Il campo purpose_of_use non è valorizzato</t>
   </si>
   <si>
-    <t>4460197c48e185eaf13de5d788bc5591</t>
-  </si>
-  <si>
     <t>Il servizio di validazione nazionale FSE non risponde</t>
   </si>
   <si>
     <t>Il sistema annulla l'operazione e consente di provare in un altro momento</t>
   </si>
   <si>
-    <t>bf17705ebe6917485589ca9767e05406</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.bb2093481e857cf61f9809da5d1e547cf570faaebdd85d80edca50144e200996.55a79aa145^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Errore semantico: [Errore-47| codice fiscale 'bscmnl99a13m172z' cittadino ed operatore: 16 cifre [A-Z0-9]{16}]</t>
   </si>
   <si>
     <t>Il sistema annulla l'operazione e consente di provare in un altro momento dopo aver corretto l'identificativo cittadino</t>
   </si>
   <si>
-    <t>935e735cd7462576542ae28ff42cd732</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.4cbd686f69c4cbf3e476e566ab542e2f95bae8897dbe4a60cf63b525dc6122e2.09e1eeb9a6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Errore semantico: [ERRORE-14| L'elemento ClinicalDocument/recordTaget/patientRole/patient/name DEVE riportare gli elementi 'given' e 'family']</t>
   </si>
   <si>
@@ -847,145 +823,166 @@
     <t>Errore semantico: Almeno uno dei seguenti vocaboli non è censito: [CodeSystem: 2.16.840.1.113883.5.1 v2.1.0, Codes: T]</t>
   </si>
   <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.477d2e947d5730e0101b6a0ac00b047a7af2d44625ba8dd5e151b9498150a5f9.be70609ba0^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>c09ebc7b268ae7702bec596907d9396c</t>
-  </si>
-  <si>
-    <t>f7100e60a4c2edcd8cf408beda26783d</t>
-  </si>
-  <si>
     <t>Errore semantico: [ERRORE-b5| Sezione Condizioni del paziente e diagnosi alla dimissione: la sezione DEVE essere presente],[ERRORE-b6| Sezione Condizioni del paziente e diagnosi alla dimissione: La sezione DEVE contenere l'elemento 'text'],[W003|  Sezione Condizioni del paziente e diagnosi alla dimissione: La sezione PUO' contenere l'elemento 'entry' ]</t>
   </si>
   <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.1ae34d558b8685de371c68b9bf4706642119e6e03fd44b2773469f989abd6597.95f15d1217^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Il sistema annulla l'operazione e consente di provare in un altro momento dopo aver corretto i dati del documento</t>
   </si>
   <si>
-    <t>9c6d793f2791fe7481a0c52eeae0754e</t>
-  </si>
-  <si>
     <t>Errore semantico: [ERRORE-b3| Sezione Decorso Ospedaliero: la sezione DEVE essere presente],[ERRORE-b4| Sezione Decorso Ospedaliero: La sezione deve contenere l'elemento 'text']</t>
   </si>
   <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.4c035ad34f501bd2c4ed9ed70ade02f81fc930e8177f0293f65d85cf766cc8e4.385a87ee23^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>9fbcde826888e3261d9a436ac7b3cea8</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.754584a7b967c83a10b8b8b7321446341181ec920634f2201186150d9b81a84e.675e64ccee^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Errore vocabolario: Almeno uno dei seguenti vocaboli non è censito: [CodeSystem: 2.16.840.1.113883.6.103, Codes: 000]</t>
   </si>
   <si>
     <t>Il sistema annulla l'operazione e consente di provare in un altro momento dopo aver corretto la diagnosi</t>
   </si>
   <si>
-    <t>dab7db01a1b7ecb923bb8919c066efb8</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.6f149c2e09c44e95b2725fd4a41d9eb5bd99e198a83f022e2bce3f5125fed0a3.ac2a64882d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Errore semantico: [ERRORE-44| Il codice fiscale 'bscmnl99a13m172z' cittadino ed operatore deve essere costituito da 16 cifre [A-Z0-9]{16}]</t>
   </si>
   <si>
-    <t>b5191ce0a1bbbd4235291c0c79729089</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.df696adef98b1f9a8cf54f0fb2524b685311a5beacbbd617c6d1cd406b2d7786.58a4a49239^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Errore semantico.:[ERRORE-14| L'elemento ClinicalDocument/recordTaget/patientRole/patient/name DEVE riportare gli elementi 'given' e 'family']</t>
   </si>
   <si>
-    <t>132cb78d7148ba0182093c71f15999a1</t>
-  </si>
-  <si>
     <t>Errore vocabolario: Almeno uno dei seguenti vocaboli non è censito: [CodeSystem: 2.16.840.1.113883.5.1 v2.1.0, Codes: T]</t>
   </si>
   <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.93798c4b5f702dc29fd9fad840ee216797712ac01d6b52075e258bb1814bdd36.fa29a0e047^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>36e399ba3189870108476e0798737eff</t>
-  </si>
-  <si>
     <t>Errore di sintassi: ERROR: -1,-1 cvc-pattern-valid: Value '' is not facet-valid with respect to pattern '[^\\s]+' for type 'cs'.,ERROR: -1,-1 cvc-attribute.3: The value '' of attribute 'code' on element 'code' is not valid with respect to its type, 'cs'.,ERROR: -1,-1 cvc-pattern-valid: Value '' is not facet-valid with respect to pattern '[^\\s]+' for type 'cs'.,ERROR: -1,-1 cvc-attribute.3: The value '' of attribute 'code' on element 'code' is not valid with respect to its type, 'cs'.</t>
   </si>
   <si>
-    <t>2bc5f166ffaf8eb25db0ebcb902ea5f4</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.77aeba502931214efd82027c63f904df6a7bee9b1fe7dfd8f918ebee1347a65d.eca9c00d39^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.c445f26f3d1056b92fb64158a079e959ae6e6b95176b68349f9676427dec4ee6.3b6ed8122d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Errore semantico: [ERRORE-b4| Sezione Referto: la sezione DEVE essere presente],[ERRORE-b5| Sezione Referto: la sezione DEVE contenere un elemento 'text']</t>
   </si>
   <si>
-    <t>5f47ef94fb7ec50ed9a26b66fa76dabd</t>
-  </si>
-  <si>
     <t>Errore semantico: [ERRORE-b6| Sezione Quesito Diagnostico: la sezione DEVE contenere un elemento 'text']</t>
   </si>
   <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.ec48ad30e5448d07e18e5f8ae8dda57e1e29bca768c3020152da9dc272b2f54c.0353d040c2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>07b415dd9f141087f104063436a91806</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.35cb19ad2901dda9ad6ecfedef2289fd0e6b48659f95d71f94405b20420ec8d3.9ad67be0ff^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Errore semantico : [ERRORE-b1| Sezione Prestazioni: la sezione DEVE essere presente]</t>
   </si>
   <si>
-    <t>036d7ddd623735b886bdc4aab34c4276</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.31ff4203e418d87aa264fe10188a56e8c300f065f76a9c64cac94a5b5a241f85.a2bca6c5e9^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Errore semantico: [ERRORE-30| L'elemento ClinicalDocument/legalAuthenticator/signatureCode deve essere valorizzato con il codice \"S\" ]</t>
   </si>
   <si>
-    <t>5f826dbfc669c773409b317611f1c7f3</t>
-  </si>
-  <si>
     <t>Errore di sintassi.:"ERROR: -1,-1 cvc-complex-type.2.4.a: Invalid content was found starting with element '{\"urn:hl7-org:v3\":languageCode}'. One of '{\"urn:hl7-org:v3\":confidentialityCode}' is expected.</t>
   </si>
   <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.bcd985527a8ae07974f89b809c25f49a217c60f4f4bc4437360b9c819cc279ee.cee45b8271^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>4ddb82f1e08dd664b4070be243cfcaf6</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.b738acf04f7eccafb1ae9e8a092932b0f8ff927c9d67b93a2aabe9396ed57c0e.bd85fd14ea^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>a50838f6cae803858d9804c56d305b9f</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.d2b1aca57ee481f1a79c7646e943a39ff77240b1dadc0a0c463b0b0739f35e1f.93d8e44eab^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>18/03/2026 110327</t>
-  </si>
-  <si>
-    <t>0c7ef65713fd9e5516762ca869f246da</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.10.639.4.4.a55f567080dde90eb939ce3a18a0a952f87b2f35411df25e15aa44509bf3b1ec.1a1b850998^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>65fa5ff0ba7d0f22266274484cf07e7f</t>
+  </si>
+  <si>
+    <t>ded2e35b75da6188c7c34364933a887a</t>
+  </si>
+  <si>
+    <t>fb75c4cdc9dd91f2e8f044fb6755e3f2</t>
+  </si>
+  <si>
+    <t>04a4addc18a668cf5d1b312f32b071c4</t>
+  </si>
+  <si>
+    <t>51ccbd32d88046920780873706cd0cab</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.429a28a4a99cef19254e6b751e0edd95eb61e90301395c2096fab47880f7b463.fad3d910c8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>5917f78584819dde93a22cdd8f8420e7</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.a78b46c16e4a008d886aace5595b1b4e703c8da7b1d3ade40ac58d9652be07ec.3271c7b9b0^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>524c9a935b252a29890679c0f3a8320f</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.7e847d79f550224a9da515d78718f8cf7ef88bf2a0477f756f689bd140322363.1660c6e056^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>3181e98d4223ef35f7e22041bbcaf8fa</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.410494f4753db83a7b2fab39eaed51dea89c4ba5aeab3bc815948bf79ca3ad0e.8fbd81e383^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>ff427983b30cc290fcda54a2548cebee</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.2a02aec657a129dc411c179b032ef20d8bf709c033fcb2169ca9c2781d8f52d4.e9fe5391c7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>5995a1af5c1bcfea167973bbd1aaf5e0</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.00fb02d540ed292e66e30ed22f21dc10e5348718ff185d9f782c95daa6b6dafd.a0c1d32f4e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>fe4727538340b44d40855e307999af12</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.b84f8852b55fc3bd56d240a94fcbb885f4740d4edaa169fe16fb7f70c496cc7a.b53a5b2c39^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>54133db3c530057efc6383adcf734d7a</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.184b420ec6a0d9100dea5b193f9cd57fcd6c46fbac5495dba84d159ab9d6113e.f32e5f86c7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>e01ad0806eb224a60c4b18e6caf0893e</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.01665aa16d720b73d009ba54ed5455ce3de15a46fce1070552df73136cfac2aa.edcb4c9efc^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>1560113c7e775e97facfaa996b8e352b</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.091050d08404e0f8346aa9722e1c6f825e266274cf72e8572cc4b360772584f4.e4d46c82c6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>44dc606b0f5f8446f12f00d6cbf0751f</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.d8ca654ca9da05f623b6fb53459e569ff108561ac68c35dec221adf3e62fc1bb.4d79e8e9c2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>f2e314876315115a4c13ab8156726c77</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.82913617651df3bddf32ca8a57b6fab91283d7d1de86f55215ceb2b6b11904d0.9312a8b1eb^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>5e98691c68a02f228b20bba4d7d5967e</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.3d62334b3d096ec4aec6a8cb0fee67a4ee707cba4fceb1b4012e5826fc895c94.0c99efba7c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>93226398f0e207aa6b1a8e2b4bdff9c6</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.e8a107f5a4c0ef378b7ebe1841a93ee7ae87e737a835c521d818aa61f66c2bae.8d73e40cdf^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>8cae4e8c06911c2351e4cc3f66a1a0fe</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.d2b1aca57ee481f1a79c7646e943a39ff77240b1dadc0a0c463b0b0739f35e1f.d87646716c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>aaece6455d6897d5ebe92dddca07b578</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.a55f567080dde90eb939ce3a18a0a952f87b2f35411df25e15aa44509bf3b1ec.6afce53ba9^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>38e0dbc8573ee65bc9db95648a5c946d</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.b738acf04f7eccafb1ae9e8a092932b0f8ff927c9d67b93a2aabe9396ed57c0e.a2b8a8d987^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>232448caedf4ecf5f5fe432bbc5d5d4c</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.10.639.4.4.0c524b55e598dc4cc98a39f57f416c7d8429a6fc35d5a8b76737b630d619e473.5034d5715d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -1486,7 +1483,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1609,12 +1606,6 @@
     <xf numFmtId="166" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1622,6 +1613,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3126,14 +3129,14 @@
       <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="55" t="s">
+      <c r="B2" s="56"/>
+      <c r="C2" s="57" t="s">
         <v>169</v>
       </c>
-      <c r="D2" s="54"/>
+      <c r="D2" s="56"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -3154,14 +3157,14 @@
       <c r="W2" s="9"/>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="62" t="s">
+      <c r="B3" s="59"/>
+      <c r="C3" s="64" t="s">
         <v>172</v>
       </c>
-      <c r="D3" s="54"/>
+      <c r="D3" s="56"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -3182,12 +3185,12 @@
       <c r="W3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="58"/>
-      <c r="B4" s="59"/>
-      <c r="C4" s="62" t="s">
+      <c r="A4" s="60"/>
+      <c r="B4" s="61"/>
+      <c r="C4" s="64" t="s">
         <v>170</v>
       </c>
-      <c r="D4" s="54"/>
+      <c r="D4" s="56"/>
       <c r="E4" s="4"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -3209,12 +3212,12 @@
       <c r="W4" s="9"/>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="60"/>
-      <c r="B5" s="61"/>
-      <c r="C5" s="63" t="s">
+      <c r="A5" s="62"/>
+      <c r="B5" s="63"/>
+      <c r="C5" s="65" t="s">
         <v>171</v>
       </c>
-      <c r="D5" s="64"/>
+      <c r="D5" s="66"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -3235,10 +3238,10 @@
       <c r="W5" s="9"/>
     </row>
     <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="51"/>
-      <c r="B6" s="52"/>
+      <c r="A6" s="53"/>
+      <c r="B6" s="54"/>
       <c r="C6" s="10"/>
-      <c r="E6" s="50"/>
+      <c r="E6" s="48"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -3389,16 +3392,16 @@
         <v>42</v>
       </c>
       <c r="F10" s="34">
-        <v>46085</v>
+        <v>46100</v>
       </c>
       <c r="G10" s="42">
-        <v>46085.423946759256</v>
+        <v>46100.378599537034</v>
       </c>
       <c r="H10" s="34" t="s">
+        <v>199</v>
+      </c>
+      <c r="I10" s="39" t="s">
         <v>173</v>
-      </c>
-      <c r="I10" s="39" t="s">
-        <v>174</v>
       </c>
       <c r="J10" s="35" t="s">
         <v>51</v>
@@ -3412,7 +3415,7 @@
         <v>51</v>
       </c>
       <c r="O10" s="43" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="P10" s="35" t="s">
         <v>51</v>
@@ -3424,7 +3427,7 @@
         <v>89</v>
       </c>
       <c r="S10" s="43" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T10" s="35" t="s">
         <v>87</v>
@@ -3452,16 +3455,16 @@
         <v>42</v>
       </c>
       <c r="F11" s="34">
-        <v>46084</v>
+        <v>46100</v>
       </c>
       <c r="G11" s="44">
-        <v>46085.37767361111</v>
+        <v>46100.383692129632</v>
       </c>
       <c r="H11" s="34" t="s">
-        <v>177</v>
+        <v>200</v>
       </c>
       <c r="I11" s="39" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J11" s="35" t="s">
         <v>51</v>
@@ -3475,7 +3478,7 @@
         <v>51</v>
       </c>
       <c r="O11" s="35" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="P11" s="35" t="s">
         <v>51</v>
@@ -3487,7 +3490,7 @@
         <v>89</v>
       </c>
       <c r="S11" s="35" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T11" s="35" t="s">
         <v>87</v>
@@ -3515,16 +3518,16 @@
         <v>48</v>
       </c>
       <c r="F12" s="34">
-        <v>46085</v>
+        <v>46100</v>
       </c>
       <c r="G12" s="44">
-        <v>46085.434687499997</v>
+        <v>46100.386111111111</v>
       </c>
       <c r="H12" s="34" t="s">
-        <v>179</v>
+        <v>201</v>
       </c>
       <c r="I12" s="39" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J12" s="35" t="s">
         <v>51</v>
@@ -3538,7 +3541,7 @@
         <v>51</v>
       </c>
       <c r="O12" s="35" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="P12" s="35" t="s">
         <v>51</v>
@@ -3550,7 +3553,7 @@
         <v>89</v>
       </c>
       <c r="S12" s="35" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T12" s="35" t="s">
         <v>87</v>
@@ -3578,16 +3581,16 @@
         <v>48</v>
       </c>
       <c r="F13" s="34">
-        <v>46084</v>
+        <v>46100</v>
       </c>
       <c r="G13" s="44">
-        <v>46084.378298611111</v>
+        <v>46100.387974537036</v>
       </c>
       <c r="H13" s="34" t="s">
-        <v>181</v>
+        <v>202</v>
       </c>
       <c r="I13" s="39" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J13" s="35" t="s">
         <v>51</v>
@@ -3601,7 +3604,7 @@
         <v>51</v>
       </c>
       <c r="O13" s="35" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="P13" s="35" t="s">
         <v>51</v>
@@ -3613,7 +3616,7 @@
         <v>89</v>
       </c>
       <c r="S13" s="35" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T13" s="35" t="s">
         <v>87</v>
@@ -3660,7 +3663,7 @@
         <v>51</v>
       </c>
       <c r="O14" s="35" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="P14" s="35" t="s">
         <v>51</v>
@@ -3672,7 +3675,7 @@
         <v>89</v>
       </c>
       <c r="S14" s="35" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="T14" s="35" t="s">
         <v>87</v>
@@ -3721,7 +3724,7 @@
         <v>51</v>
       </c>
       <c r="O15" s="35" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="P15" s="35" t="s">
         <v>51</v>
@@ -3733,7 +3736,7 @@
         <v>89</v>
       </c>
       <c r="S15" s="35" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="T15" s="35" t="s">
         <v>87</v>
@@ -3763,16 +3766,16 @@
         <v>115</v>
       </c>
       <c r="F16" s="34">
-        <v>46085</v>
+        <v>46100</v>
       </c>
       <c r="G16" s="44">
-        <v>46085.443796296298</v>
+        <v>46100.391180555554</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>184</v>
+        <v>203</v>
       </c>
       <c r="I16" s="39" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="J16" s="35" t="s">
         <v>51</v>
@@ -3786,7 +3789,7 @@
         <v>51</v>
       </c>
       <c r="O16" s="35" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="P16" s="35" t="s">
         <v>51</v>
@@ -3798,7 +3801,7 @@
         <v>89</v>
       </c>
       <c r="S16" s="35" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="T16" s="35" t="s">
         <v>87</v>
@@ -3859,20 +3862,20 @@
       <c r="D18" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="E18" s="40" t="s">
+      <c r="E18" s="49" t="s">
         <v>117</v>
       </c>
       <c r="F18" s="34">
-        <v>46085</v>
+        <v>46100</v>
       </c>
       <c r="G18" s="44">
-        <v>46085.464884259258</v>
+        <v>46100.393877314818</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>188</v>
+        <v>205</v>
       </c>
       <c r="I18" s="39" t="s">
-        <v>189</v>
+        <v>206</v>
       </c>
       <c r="J18" s="35" t="s">
         <v>51</v>
@@ -3886,7 +3889,7 @@
         <v>51</v>
       </c>
       <c r="O18" s="35" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="P18" s="35" t="s">
         <v>51</v>
@@ -3898,7 +3901,7 @@
         <v>89</v>
       </c>
       <c r="S18" s="35" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="T18" s="35" t="s">
         <v>87</v>
@@ -3926,16 +3929,16 @@
         <v>118</v>
       </c>
       <c r="F19" s="34">
-        <v>46085</v>
+        <v>46100</v>
       </c>
       <c r="G19" s="44">
-        <v>46085.465925925928</v>
+        <v>46100.398912037039</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="I19" s="39" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="J19" s="35" t="s">
         <v>51</v>
@@ -3949,7 +3952,7 @@
         <v>51</v>
       </c>
       <c r="O19" s="35" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="P19" s="35" t="s">
         <v>51</v>
@@ -3961,7 +3964,7 @@
         <v>89</v>
       </c>
       <c r="S19" s="35" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="T19" s="35" t="s">
         <v>87</v>
@@ -3989,16 +3992,16 @@
         <v>119</v>
       </c>
       <c r="F20" s="34">
-        <v>46085</v>
+        <v>46100</v>
       </c>
       <c r="G20" s="44">
-        <v>46085.466412037036</v>
+        <v>46100.401886574073</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="I20" s="39" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="J20" s="35" t="s">
         <v>51</v>
@@ -4012,7 +4015,7 @@
         <v>51</v>
       </c>
       <c r="O20" s="35" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="P20" s="35" t="s">
         <v>51</v>
@@ -4024,7 +4027,7 @@
         <v>89</v>
       </c>
       <c r="S20" s="35" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="T20" s="35" t="s">
         <v>87</v>
@@ -4052,16 +4055,16 @@
         <v>120</v>
       </c>
       <c r="F21" s="34">
-        <v>46085</v>
+        <v>46100</v>
       </c>
       <c r="G21" s="44">
-        <v>46085.484953703701</v>
+        <v>46100.404270833336</v>
       </c>
       <c r="H21" s="34" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="I21" s="39" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="J21" s="35" t="s">
         <v>51</v>
@@ -4074,7 +4077,7 @@
         <v>51</v>
       </c>
       <c r="O21" s="35" t="s">
-        <v>200</v>
+        <v>187</v>
       </c>
       <c r="P21" s="35" t="s">
         <v>51</v>
@@ -4086,7 +4089,7 @@
         <v>89</v>
       </c>
       <c r="S21" s="35" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="T21" s="35" t="s">
         <v>87</v>
@@ -4196,16 +4199,16 @@
         <v>123</v>
       </c>
       <c r="F24" s="34">
-        <v>46085</v>
+        <v>46100</v>
       </c>
       <c r="G24" s="44">
-        <v>46085.561273148145</v>
+        <v>46100.406840277778</v>
       </c>
       <c r="H24" s="34" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="I24" s="39" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="J24" s="35" t="s">
         <v>51</v>
@@ -4219,7 +4222,7 @@
         <v>51</v>
       </c>
       <c r="O24" s="35" t="s">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="P24" s="35" t="s">
         <v>51</v>
@@ -4231,7 +4234,7 @@
         <v>89</v>
       </c>
       <c r="S24" s="35" t="s">
-        <v>205</v>
+        <v>189</v>
       </c>
       <c r="T24" s="35" t="s">
         <v>87</v>
@@ -4300,16 +4303,16 @@
         <v>125</v>
       </c>
       <c r="F26" s="34">
-        <v>46084</v>
+        <v>46100</v>
       </c>
       <c r="G26" s="44">
-        <v>46084.421747685185</v>
+        <v>46100.410057870373</v>
       </c>
       <c r="H26" s="34" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="I26" s="39" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="J26" s="35" t="s">
         <v>51</v>
@@ -4323,7 +4326,7 @@
         <v>51</v>
       </c>
       <c r="O26" s="35" t="s">
-        <v>208</v>
+        <v>190</v>
       </c>
       <c r="P26" s="35" t="s">
         <v>51</v>
@@ -4335,7 +4338,7 @@
         <v>89</v>
       </c>
       <c r="S26" s="35" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="T26" s="35" t="s">
         <v>87</v>
@@ -4364,7 +4367,7 @@
       </c>
       <c r="F27" s="34"/>
       <c r="G27" s="44"/>
-      <c r="H27" s="49"/>
+      <c r="H27" s="47"/>
       <c r="I27" s="39"/>
       <c r="J27" s="35" t="s">
         <v>89</v>
@@ -4404,16 +4407,16 @@
         <v>127</v>
       </c>
       <c r="F28" s="34">
-        <v>46084</v>
+        <v>46100</v>
       </c>
       <c r="G28" s="44">
-        <v>46084.489131944443</v>
+        <v>46100.415891203702</v>
       </c>
       <c r="H28" s="34" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="I28" s="39" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="J28" s="35" t="s">
         <v>51</v>
@@ -4427,7 +4430,7 @@
         <v>51</v>
       </c>
       <c r="O28" s="35" t="s">
-        <v>211</v>
+        <v>191</v>
       </c>
       <c r="P28" s="35" t="s">
         <v>51</v>
@@ -4439,7 +4442,7 @@
         <v>89</v>
       </c>
       <c r="S28" s="35" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="T28" s="35" t="s">
         <v>87</v>
@@ -4467,16 +4470,16 @@
         <v>128</v>
       </c>
       <c r="F29" s="34">
-        <v>46084</v>
+        <v>46100</v>
       </c>
       <c r="G29" s="44">
-        <v>46084.490219907406</v>
+        <v>46100.421018518522</v>
       </c>
       <c r="H29" s="34" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="I29" s="39" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="J29" s="35" t="s">
         <v>51</v>
@@ -4490,7 +4493,7 @@
         <v>51</v>
       </c>
       <c r="O29" s="35" t="s">
-        <v>213</v>
+        <v>192</v>
       </c>
       <c r="P29" s="35" t="s">
         <v>51</v>
@@ -4502,7 +4505,7 @@
         <v>89</v>
       </c>
       <c r="S29" s="35" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="T29" s="35" t="s">
         <v>87</v>
@@ -4571,16 +4574,16 @@
         <v>71</v>
       </c>
       <c r="F31" s="34">
-        <v>46084</v>
+        <v>46100</v>
       </c>
       <c r="G31" s="44">
-        <v>46084.491342592592</v>
+        <v>46100.442824074074</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="I31" s="39" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="J31" s="35" t="s">
         <v>51</v>
@@ -4594,7 +4597,7 @@
         <v>51</v>
       </c>
       <c r="O31" s="35" t="s">
-        <v>216</v>
+        <v>193</v>
       </c>
       <c r="P31" s="35" t="s">
         <v>51</v>
@@ -4606,7 +4609,7 @@
         <v>89</v>
       </c>
       <c r="S31" s="35" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="T31" s="35" t="s">
         <v>87</v>
@@ -4634,16 +4637,16 @@
         <v>106</v>
       </c>
       <c r="F32" s="34">
-        <v>46084</v>
+        <v>46100</v>
       </c>
       <c r="G32" s="44">
-        <v>46084.493148148147</v>
+        <v>46100.444687499999</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="I32" s="39" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="J32" s="35" t="s">
         <v>51</v>
@@ -4657,7 +4660,7 @@
         <v>51</v>
       </c>
       <c r="O32" s="35" t="s">
-        <v>220</v>
+        <v>194</v>
       </c>
       <c r="P32" s="35" t="s">
         <v>51</v>
@@ -4669,7 +4672,7 @@
         <v>89</v>
       </c>
       <c r="S32" s="35" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="T32" s="35" t="s">
         <v>87</v>
@@ -4697,16 +4700,16 @@
         <v>107</v>
       </c>
       <c r="F33" s="34">
-        <v>46084</v>
+        <v>46100</v>
       </c>
       <c r="G33" s="44">
-        <v>46084.494039351855</v>
+        <v>46100.452118055553</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I33" s="39" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="J33" s="35" t="s">
         <v>51</v>
@@ -4720,7 +4723,7 @@
         <v>51</v>
       </c>
       <c r="O33" s="35" t="s">
-        <v>222</v>
+        <v>195</v>
       </c>
       <c r="P33" s="35" t="s">
         <v>51</v>
@@ -4732,7 +4735,7 @@
         <v>89</v>
       </c>
       <c r="S33" s="35" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="T33" s="35" t="s">
         <v>87</v>
@@ -4760,16 +4763,16 @@
         <v>108</v>
       </c>
       <c r="F34" s="34">
-        <v>46084</v>
+        <v>46100</v>
       </c>
       <c r="G34" s="44">
-        <v>46084.494710648149</v>
+        <v>46100.456724537034</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="I34" s="39" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="J34" s="35" t="s">
         <v>51</v>
@@ -4783,7 +4786,7 @@
         <v>51</v>
       </c>
       <c r="O34" s="35" t="s">
-        <v>226</v>
+        <v>196</v>
       </c>
       <c r="P34" s="35" t="s">
         <v>51</v>
@@ -4795,7 +4798,7 @@
         <v>89</v>
       </c>
       <c r="S34" s="35" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="T34" s="35" t="s">
         <v>87</v>
@@ -5028,16 +5031,16 @@
         <v>114</v>
       </c>
       <c r="F40" s="34">
-        <v>46084</v>
+        <v>46100</v>
       </c>
       <c r="G40" s="39">
-        <v>46084.495636574073</v>
-      </c>
-      <c r="H40" s="46" t="s">
-        <v>227</v>
-      </c>
-      <c r="I40" s="47" t="s">
-        <v>228</v>
+        <v>46100.459027777775</v>
+      </c>
+      <c r="H40" s="50" t="s">
+        <v>237</v>
+      </c>
+      <c r="I40" s="52" t="s">
+        <v>238</v>
       </c>
       <c r="J40" s="35" t="s">
         <v>51</v>
@@ -5051,7 +5054,7 @@
         <v>51</v>
       </c>
       <c r="O40" s="35" t="s">
-        <v>229</v>
+        <v>197</v>
       </c>
       <c r="P40" s="35" t="s">
         <v>51</v>
@@ -5063,7 +5066,7 @@
         <v>89</v>
       </c>
       <c r="S40" s="35" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="T40" s="35" t="s">
         <v>87</v>
@@ -5091,16 +5094,16 @@
         <v>140</v>
       </c>
       <c r="F41" s="34">
-        <v>46090</v>
+        <v>46100</v>
       </c>
       <c r="G41" s="44">
-        <v>46090.459652777776</v>
+        <v>46100.563090277778</v>
       </c>
       <c r="H41" s="34" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I41" s="39" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="J41" s="35" t="s">
         <v>51</v>
@@ -5176,16 +5179,16 @@
         <v>136</v>
       </c>
       <c r="F43" s="34">
-        <v>46098</v>
+        <v>46100</v>
       </c>
       <c r="G43" s="44">
-        <v>46098.422615740739</v>
+        <v>46100.51221064815</v>
       </c>
       <c r="H43" s="34" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="I43" s="39" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="J43" s="35" t="s">
         <v>51</v>
@@ -5225,16 +5228,16 @@
         <v>137</v>
       </c>
       <c r="F44" s="34">
-        <v>46099</v>
-      </c>
-      <c r="G44" s="44" t="s">
-        <v>237</v>
+        <v>46100</v>
+      </c>
+      <c r="G44" s="44">
+        <v>46100.513935185183</v>
       </c>
       <c r="H44" s="34" t="s">
-        <v>238</v>
-      </c>
-      <c r="I44" s="39" t="s">
-        <v>239</v>
+        <v>233</v>
+      </c>
+      <c r="I44" s="51" t="s">
+        <v>234</v>
       </c>
       <c r="J44" s="35" t="s">
         <v>51</v>
@@ -5314,17 +5317,17 @@
       <c r="E46" s="40" t="s">
         <v>147</v>
       </c>
-      <c r="F46" s="48">
-        <v>46085</v>
+      <c r="F46" s="46">
+        <v>46100</v>
       </c>
       <c r="G46" s="45">
-        <v>46085.563715277778</v>
+        <v>46100.483553240738</v>
       </c>
       <c r="H46" s="35" t="s">
+        <v>229</v>
+      </c>
+      <c r="I46" s="35" t="s">
         <v>230</v>
-      </c>
-      <c r="I46" s="35" t="s">
-        <v>232</v>
       </c>
       <c r="J46" s="35" t="s">
         <v>51</v>
@@ -5338,7 +5341,7 @@
         <v>51</v>
       </c>
       <c r="O46" s="35" t="s">
-        <v>231</v>
+        <v>198</v>
       </c>
       <c r="P46" s="35" t="s">
         <v>51</v>
@@ -5350,7 +5353,7 @@
         <v>89</v>
       </c>
       <c r="S46" s="35" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="T46" s="35" t="s">
         <v>87</v>

</xml_diff>